<commit_message>
docs: cap nhat Sprint Planning 1-3 va Product Backlog cho khop thuc te
US-13 'Done' -> chuyen Sprint 3; Sprint 3: US-13, US-14, US-15 ve To Do (chua co ma nguon). Cot cong nghe theo thuc te (node:test, Expo, Playwright, Maestro). Product Backlog them cot Sprint/Story, trang thai, ghi chu; sua ten bi dich may (ghi lai ten cu); Sprint Backlog: US-26 lam som, muc 'Ngoai ke hoach'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ProductBacklog-nhom17.xlsx
+++ b/docs/ProductBacklog-nhom17.xlsx
@@ -18,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -871,7 +872,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -953,6 +954,21 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1650,6 +1666,9 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="67.2685185185185" customWidth="1" min="2" max="2"/>
     <col width="6.12962962962963" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.4" customHeight="1">
@@ -1680,11 +1699,29 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>Sprint / Story</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="inlineStr">
+        <is>
+          <t>Trạng thái 29/10/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="13.95" customHeight="1">
       <c r="A4" s="19" t="n"/>
       <c r="B4" s="15" t="n"/>
       <c r="C4" s="20" t="n"/>
+      <c r="D4" s="20" t="n"/>
+      <c r="E4" s="49" t="n"/>
+      <c r="F4" s="49" t="n"/>
     </row>
     <row r="5" ht="15.6" customHeight="1">
       <c r="A5" s="21" t="n"/>
@@ -1694,6 +1731,9 @@
         </is>
       </c>
       <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="50" t="n"/>
+      <c r="F5" s="50" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="24" t="n">
@@ -1707,6 +1747,17 @@
       <c r="C6" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>PB-01 · làm sớm</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>Done (mức xem)</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="24" t="n">
@@ -1720,6 +1771,17 @@
       <c r="C7" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>US-22 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E7" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F7" s="51" t="n"/>
       <c r="G7" s="27" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -1734,6 +1796,17 @@
       <c r="C8" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>US-16 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="n"/>
       <c r="H8" s="26" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -1748,6 +1821,17 @@
       <c r="C9" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>PB-04 · làm sớm</t>
+        </is>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>Done (mức xem)</t>
+        </is>
+      </c>
+      <c r="F9" s="51" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="24" t="n">
@@ -1761,6 +1845,17 @@
       <c r="C10" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>US-07 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E10" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F10" s="51" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="24" t="n">
@@ -1774,7 +1869,17 @@
       <c r="C11" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="26" t="n"/>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>US-06 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E11" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="51" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="24" t="n">
@@ -1788,6 +1893,17 @@
       <c r="C12" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="n"/>
     </row>
     <row r="13" ht="15.6" customHeight="1">
       <c r="A13" s="21" t="n"/>
@@ -1797,6 +1913,9 @@
         </is>
       </c>
       <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="50" t="n"/>
+      <c r="F13" s="50" t="n"/>
       <c r="G13" s="26" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -1811,6 +1930,17 @@
       <c r="C14" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>US-08 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E14" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="51" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="24" t="n">
@@ -1824,6 +1954,17 @@
       <c r="C15" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F15" s="51" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="24" t="n">
@@ -1837,6 +1978,17 @@
       <c r="C16" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>US-15 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E16" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F16" s="51" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="24" t="n">
@@ -1844,11 +1996,26 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>Update hồ sơ cá nhân và cửa hàng thông tin</t>
+          <t>Cập nhật hồ sơ cá nhân và thông tin cửa hàng</t>
         </is>
       </c>
       <c r="C17" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F17" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Update hồ sơ cá nhân và cửa hàng thông tin”)</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1863,6 +2030,17 @@
       <c r="C18" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F18" s="51" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="24" t="n">
@@ -1876,6 +2054,17 @@
       <c r="C19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>US-18 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E19" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F19" s="51" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="24" t="n">
@@ -1889,6 +2078,17 @@
       <c r="C20" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>US-17 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E20" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F20" s="51" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="24" t="n">
@@ -1902,6 +2102,17 @@
       <c r="C21" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>US-19 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E21" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F21" s="51" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="24" t="n">
@@ -1915,6 +2126,17 @@
       <c r="C22" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F22" s="51" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="24" t="n">
@@ -1928,6 +2150,17 @@
       <c r="C23" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>US-20 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E23" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F23" s="51" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="24" t="n">
@@ -1941,6 +2174,17 @@
       <c r="C24" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="51" t="inlineStr">
+        <is>
+          <t>Release 1.1 (đã cắt)</t>
+        </is>
+      </c>
+      <c r="F24" s="51" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="24" t="n">
@@ -1954,6 +2198,17 @@
       <c r="C25" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F25" s="51" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="24" t="n">
@@ -1967,6 +2222,17 @@
       <c r="C26" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="51" t="inlineStr">
+        <is>
+          <t>Release 1.1 (đã cắt)</t>
+        </is>
+      </c>
+      <c r="F26" s="51" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="24" t="n">
@@ -1974,11 +2240,26 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>Xem danh sách và chi tiết bất kỳ đối thoại</t>
+          <t>Xem danh sách và chi tiết kỳ đối soát</t>
         </is>
       </c>
       <c r="C27" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F27" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem danh sách và chi tiết bất kỳ đối thoại”)</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1987,11 +2268,26 @@
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>Hủy đơn hàng khi chưa nhận được</t>
+          <t>Hủy đơn hàng khi chưa được lấy hàng</t>
         </is>
       </c>
       <c r="C28" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F28" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Hủy đơn hàng khi chưa nhận được”)</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2000,11 +2296,26 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>Chỉnh sửa đơn hàng khi chưa lấy được</t>
+          <t>Chỉnh sửa đơn hàng khi chưa lấy hàng</t>
         </is>
       </c>
       <c r="C29" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F29" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Chỉnh sửa đơn hàng khi chưa lấy được”)</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2013,11 +2324,26 @@
       </c>
       <c r="B30" s="25" t="inlineStr">
         <is>
-          <t>Yêu cầu lại đối với đơn vị thất bại</t>
+          <t>Yêu cầu giao lại đối với đơn giao thất bại</t>
         </is>
       </c>
       <c r="C30" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F30" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Yêu cầu lại đối với đơn vị thất bại”)</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2026,11 +2352,26 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>Tạo yêu cầu hỗ trợ hoặc giải nén cho một hàng</t>
+          <t>Tạo yêu cầu hỗ trợ hoặc khiếu nại cho một đơn hàng</t>
         </is>
       </c>
       <c r="C31" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F31" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Tạo yêu cầu hỗ trợ hoặc giải nén cho một hàng”)</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2039,11 +2380,26 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>Theo dõi trạng thái xử lý xuất</t>
+          <t>Theo dõi trạng thái xử lý khiếu nại</t>
         </is>
       </c>
       <c r="C32" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F32" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Theo dõi trạng thái xử lý xuất”)</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2058,6 +2414,17 @@
       <c r="C33" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F33" s="51" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="24" t="n">
@@ -2065,11 +2432,26 @@
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>Xuất báo cáo đối thoại ra file Excel</t>
+          <t>Xuất báo cáo đối soát ra file Excel</t>
         </is>
       </c>
       <c r="C34" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F34" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xuất báo cáo đối thoại ra file Excel”)</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2084,6 +2466,17 @@
       <c r="C35" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E35" s="51" t="inlineStr">
+        <is>
+          <t>Release 1.1 (đã cắt)</t>
+        </is>
+      </c>
+      <c r="F35" s="51" t="n"/>
     </row>
     <row r="36" ht="15.6" customHeight="1">
       <c r="A36" s="28" t="n"/>
@@ -2093,6 +2486,9 @@
         </is>
       </c>
       <c r="C36" s="28" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="52" t="n"/>
+      <c r="F36" s="52" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="24" t="n">
@@ -2106,6 +2502,17 @@
       <c r="C37" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>US-26 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E37" s="51" t="inlineStr">
+        <is>
+          <t>Done (làm sớm 22/10)</t>
+        </is>
+      </c>
+      <c r="F37" s="51" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="24" t="n">
@@ -2119,6 +2526,17 @@
       <c r="C38" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>US-27 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E38" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F38" s="51" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="24" t="n">
@@ -2132,6 +2550,17 @@
       <c r="C39" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F39" s="51" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="24" t="n">
@@ -2145,6 +2574,17 @@
       <c r="C40" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>US-28 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E40" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F40" s="51" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="24" t="n">
@@ -2152,11 +2592,26 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>Ghi nhận khi không nhận được hàng</t>
+          <t>Ghi nhận khi không lấy được hàng</t>
         </is>
       </c>
       <c r="C41" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F41" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Ghi nhận khi không nhận được hàng”)</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2165,11 +2620,26 @@
       </c>
       <c r="B42" s="25" t="inlineStr">
         <is>
-          <t>Bàn giao hàng về điểm tập tin</t>
+          <t>Bàn giao hàng về điểm tập kết</t>
         </is>
       </c>
       <c r="C42" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F42" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Bàn giao hàng về điểm tập tin”)</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
@@ -2184,6 +2654,17 @@
       <c r="C43" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>US-31 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E43" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F43" s="51" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="24" t="n">
@@ -2197,6 +2678,17 @@
       <c r="C44" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D44" s="24" t="inlineStr">
+        <is>
+          <t>US-30 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E44" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F44" s="51" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="24" t="n">
@@ -2210,6 +2702,17 @@
       <c r="C45" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>US-32 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E45" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F45" s="51" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="24" t="n">
@@ -2223,6 +2726,17 @@
       <c r="C46" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>US-33 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E46" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F46" s="51" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="24" t="n">
@@ -2236,6 +2750,17 @@
       <c r="C47" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F47" s="51" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="24" t="n">
@@ -2243,11 +2768,26 @@
       </c>
       <c r="B48" s="25" t="inlineStr">
         <is>
-          <t>Chụp ảnh bằng giao dịch</t>
+          <t>Chụp ảnh bằng chứng giao hàng</t>
         </is>
       </c>
       <c r="C48" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F48" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Chụp ảnh bằng giao dịch”)</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -2256,11 +2796,26 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>Tổng hợp và trả tiền COD cuối cùng</t>
+          <t>Tổng hợp và nộp tiền COD cuối ca</t>
         </is>
       </c>
       <c r="C49" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F49" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Tổng hợp và trả tiền COD cuối cùng”)</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
@@ -2269,11 +2824,26 @@
       </c>
       <c r="B50" s="25" t="inlineStr">
         <is>
-          <t>Xác nhận đã hoàn tất hàng gửi cho người gửi</t>
+          <t>Xác nhận đã hoàn trả hàng cho người gửi</t>
         </is>
       </c>
       <c r="C50" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>US-37 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E50" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F50" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xác nhận đã hoàn tất hàng gửi cho người gửi”)</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
@@ -2282,11 +2852,26 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>Xem lịch làm việc và tuyến đường được phân tích</t>
+          <t>Xem lịch làm việc và tuyến đường được phân công</t>
         </is>
       </c>
       <c r="C51" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F51" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem lịch làm việc và tuyến đường được phân tích”)</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
@@ -2295,21 +2880,43 @@
       </c>
       <c r="B52" s="25" t="inlineStr">
         <is>
-          <t>Báo cáo sự cố phát hiện trong quá trình chuyển đổi</t>
+          <t>Báo cáo sự cố phát hiện trong quá trình vận chuyển</t>
         </is>
       </c>
       <c r="C52" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D52" s="24" t="inlineStr">
+        <is>
+          <t>US-38 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E52" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F52" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Báo cáo sự cố phát hiện trong quá trình chuyển đổi”)</t>
+        </is>
       </c>
     </row>
     <row r="53" ht="15.6" customHeight="1">
       <c r="A53" s="28" t="n"/>
       <c r="B53" s="29" t="inlineStr">
         <is>
-          <t>Là nhân viên duyệt tại cửa hàng tôi muốn</t>
+          <t>Là nhân viên tại điểm tập kết (hub) tôi muốn</t>
         </is>
       </c>
       <c r="C53" s="28" t="n"/>
+      <c r="D53" s="28" t="n"/>
+      <c r="E53" s="52" t="n"/>
+      <c r="F53" s="52" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Là nhân viên duyệt tại cửa hàng tôi muốn”)</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="24" t="n">
@@ -2317,11 +2924,26 @@
       </c>
       <c r="B54" s="25" t="inlineStr">
         <is>
-          <t>Đăng nhập và xem tổng quan điểm tinh thần</t>
+          <t>Đăng nhập và xem tổng quan điểm tập kết</t>
         </is>
       </c>
       <c r="C54" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F54" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Đăng nhập và xem tổng quan điểm tinh thần”)</t>
+        </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
@@ -2336,6 +2958,17 @@
       <c r="C55" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F55" s="51" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="24" t="n">
@@ -2349,6 +2982,17 @@
       <c r="C56" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D56" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F56" s="51" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="24" t="n">
@@ -2356,11 +3000,26 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>Duyệt đơn hàng mới được phát trong khu vực</t>
+          <t>Duyệt đơn hàng mới phát sinh trong khu vực</t>
         </is>
       </c>
       <c r="C57" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D57" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F57" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Duyệt đơn hàng mới được phát trong khu vực”)</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
@@ -2375,6 +3034,17 @@
       <c r="C58" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F58" s="51" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="24" t="n">
@@ -2388,6 +3058,17 @@
       <c r="C59" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D59" s="24" t="inlineStr">
+        <is>
+          <t>US-25 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E59" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F59" s="51" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="24" t="n">
@@ -2395,11 +3076,26 @@
       </c>
       <c r="B60" s="25" t="inlineStr">
         <is>
-          <t>Phân chia công đơn đơn hàng cho người giao hàng</t>
+          <t>Phân công đơn giao hàng cho người giao hàng</t>
         </is>
       </c>
       <c r="C60" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D60" s="24" t="inlineStr">
+        <is>
+          <t>US-35 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E60" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F60" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Phân chia công đơn đơn hàng cho người giao hàng”)</t>
+        </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
@@ -2408,11 +3104,26 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>Điều chỉnh phân tích khi có vấn đề phát sinh</t>
+          <t>Điều chỉnh phân công khi có vấn đề phát sinh</t>
         </is>
       </c>
       <c r="C61" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D61" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F61" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Điều chỉnh phân tích khi có vấn đề phát sinh”)</t>
+        </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
@@ -2421,11 +3132,26 @@
       </c>
       <c r="B62" s="25" t="inlineStr">
         <is>
-          <t>Nhập kho sự kiện khi hàng về điểm</t>
+          <t>Nhập kho kiện hàng khi hàng về điểm</t>
         </is>
       </c>
       <c r="C62" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D62" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F62" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Nhập kho sự kiện khi hàng về điểm”)</t>
+        </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
@@ -2434,11 +3160,26 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>Xuất kho và giao hàng bàn cho sản phẩm tiếp theo</t>
+          <t>Xuất kho và bàn giao hàng cho chặng tiếp theo</t>
         </is>
       </c>
       <c r="C63" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D63" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F63" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xuất kho và giao hàng bàn cho sản phẩm tiếp theo”)</t>
+        </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
@@ -2447,11 +3188,26 @@
       </c>
       <c r="B64" s="25" t="inlineStr">
         <is>
-          <t>Đã nhận và đối chiếu tiền COD do người giao hàng trả tiền</t>
+          <t>Nhận và đối chiếu tiền COD do người giao hàng nộp</t>
         </is>
       </c>
       <c r="C64" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D64" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F64" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Đã nhận và đối chiếu tiền COD do người giao hàng trả tiền”)</t>
+        </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
@@ -2460,11 +3216,26 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>Ra quyết định hoàn thành người gửi</t>
+          <t>Ra quyết định hoàn hàng cho người gửi</t>
         </is>
       </c>
       <c r="C65" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D65" s="24" t="inlineStr">
+        <is>
+          <t>US-37 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E65" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F65" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Ra quyết định hoàn thành người gửi”)</t>
+        </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
@@ -2473,11 +3244,26 @@
       </c>
       <c r="B66" s="25" t="inlineStr">
         <is>
-          <t>Xem trạng thái tải công việc của từng giao hàng</t>
+          <t>Xem tải công việc của từng người giao hàng</t>
         </is>
       </c>
       <c r="C66" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F66" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem trạng thái tải công việc của từng giao hàng”)</t>
+        </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
@@ -2486,11 +3272,26 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>Xem danh sách sự kiện đang tồn tại tại điểm</t>
+          <t>Xem danh sách kiện hàng đang tồn tại điểm</t>
         </is>
       </c>
       <c r="C67" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D67" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F67" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem danh sách sự kiện đang tồn tại tại điểm”)</t>
+        </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
@@ -2505,6 +3306,17 @@
       <c r="C68" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D68" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F68" s="51" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="24" t="n">
@@ -2512,11 +3324,26 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>Ghi nhận lỗi hoặc lỗi tại điểm</t>
+          <t>Ghi nhận sự cố hoặc khiếu nại tại điểm</t>
         </is>
       </c>
       <c r="C69" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D69" s="24" t="inlineStr">
+        <is>
+          <t>US-38 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E69" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F69" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Ghi nhận lỗi hoặc lỗi tại điểm”)</t>
+        </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
@@ -2525,11 +3352,26 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>Xử lý và cập nhật kết quả khai thác thuộc phạm vi điểm</t>
+          <t>Xử lý và cập nhật kết quả khiếu nại thuộc phạm vi điểm</t>
         </is>
       </c>
       <c r="C70" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D70" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F70" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xử lý và cập nhật kết quả khai thác thuộc phạm vi điểm”)</t>
+        </is>
       </c>
     </row>
     <row r="71" ht="15.6" customHeight="1">
@@ -2540,6 +3382,9 @@
         </is>
       </c>
       <c r="C71" s="28" t="n"/>
+      <c r="D71" s="28" t="n"/>
+      <c r="E71" s="52" t="n"/>
+      <c r="F71" s="52" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="24" t="n">
@@ -2553,6 +3398,17 @@
       <c r="C72" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D72" s="24" t="inlineStr">
+        <is>
+          <t>US-09 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E72" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F72" s="51" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="24" t="n">
@@ -2566,6 +3422,17 @@
       <c r="C73" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D73" s="24" t="inlineStr">
+        <is>
+          <t>US-10 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E73" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F73" s="51" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="24" t="n">
@@ -2579,6 +3446,17 @@
       <c r="C74" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>US-11 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E74" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F74" s="51" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="24" t="n">
@@ -2592,6 +3470,17 @@
       <c r="C75" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>US-13 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E75" s="51" t="inlineStr">
+        <is>
+          <t>To Do (chuyển từ Sprint 2)</t>
+        </is>
+      </c>
+      <c r="F75" s="51" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="24" t="n">
@@ -2605,6 +3494,17 @@
       <c r="C76" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D76" s="24" t="inlineStr">
+        <is>
+          <t>US-23 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E76" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F76" s="51" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="24" t="n">
@@ -2618,6 +3518,17 @@
       <c r="C77" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>US-14 · Sprint 3</t>
+        </is>
+      </c>
+      <c r="E77" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F77" s="51" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="24" t="n">
@@ -2631,6 +3542,17 @@
       <c r="C78" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>US-12 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E78" s="51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F78" s="51" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="24" t="n">
@@ -2638,11 +3560,26 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>Quản lý quy định danh mục bằng cách đóng gói</t>
+          <t>Quản lý danh mục quy cách đóng gói</t>
         </is>
       </c>
       <c r="C79" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D79" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F79" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Quản lý quy định danh mục bằng cách đóng gói”)</t>
+        </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
@@ -2657,6 +3594,17 @@
       <c r="C80" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>US-29 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E80" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F80" s="51" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="24" t="n">
@@ -2670,6 +3618,17 @@
       <c r="C81" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>US-10 · Sprint 2</t>
+        </is>
+      </c>
+      <c r="E81" s="51" t="inlineStr">
+        <is>
+          <t>Một phần: admin đổi PENDING → ACTIVE</t>
+        </is>
+      </c>
+      <c r="F81" s="51" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="24" t="n">
@@ -2683,6 +3642,17 @@
       <c r="C82" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>US-24 · Sprint 4</t>
+        </is>
+      </c>
+      <c r="E82" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F82" s="51" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="24" t="n">
@@ -2696,6 +3666,17 @@
       <c r="C83" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D83" s="24" t="inlineStr">
+        <is>
+          <t>US-34 · Sprint 5</t>
+        </is>
+      </c>
+      <c r="E83" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F83" s="51" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="24" t="n">
@@ -2709,6 +3690,17 @@
       <c r="C84" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F84" s="51" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="24" t="n">
@@ -2716,11 +3708,26 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>Thêm điều chỉnh tăng hoặc giảm vào bất kỳ đối số nào</t>
+          <t>Thêm điều chỉnh tăng hoặc giảm vào kỳ đối soát</t>
         </is>
       </c>
       <c r="C85" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="51" t="inlineStr">
+        <is>
+          <t>Chưa xếp Sprint</t>
+        </is>
+      </c>
+      <c r="F85" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Thêm điều chỉnh tăng hoặc giảm vào bất kỳ đối số nào”)</t>
+        </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
@@ -2729,11 +3736,26 @@
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>Cấu hình chính sách giao tiếp lại và hoàn thành điều kiện</t>
+          <t>Cấu hình chính sách giao lại và điều kiện hoàn hàng</t>
         </is>
       </c>
       <c r="C86" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="D86" s="24" t="inlineStr">
+        <is>
+          <t>US-36 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E86" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F86" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Cấu hình chính sách giao tiếp lại và hoàn thành điều kiện”)</t>
+        </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
@@ -2748,6 +3770,17 @@
       <c r="C87" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="D87" s="24" t="inlineStr">
+        <is>
+          <t>US-39 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E87" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F87" s="51" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="24" t="n">
@@ -2761,6 +3794,17 @@
       <c r="C88" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="D88" s="24" t="inlineStr">
+        <is>
+          <t>US-39 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E88" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F88" s="51" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="24" t="n">
@@ -2768,11 +3812,26 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>Xem báo cáo hiệu suất của giao dịch</t>
+          <t>Xem báo cáo hiệu suất của người giao hàng</t>
         </is>
       </c>
       <c r="C89" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>US-39 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E89" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F89" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem báo cáo hiệu suất của giao dịch”)</t>
+        </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
@@ -2781,11 +3840,26 @@
       </c>
       <c r="B90" s="25" t="inlineStr">
         <is>
-          <t>Xem báo cáo thu phí vận hành theo kỳ</t>
+          <t>Xem báo cáo doanh thu phí vận chuyển theo kỳ</t>
         </is>
       </c>
       <c r="C90" s="24" t="n">
         <v>3</v>
+      </c>
+      <c r="D90" s="24" t="inlineStr">
+        <is>
+          <t>US-39 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E90" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F90" s="51" t="inlineStr">
+        <is>
+          <t>Sửa tên 29/10/2026 (bản cũ: “Xem báo cáo thu phí vận hành theo kỳ”)</t>
+        </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
@@ -2800,6 +3874,17 @@
       <c r="C91" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="D91" s="24" t="inlineStr">
+        <is>
+          <t>US-39 · Sprint 6</t>
+        </is>
+      </c>
+      <c r="E91" s="51" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F91" s="51" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2813,7 +3898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.861111111111111" defaultRowHeight="13.2"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3276,7 +4361,7 @@
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Sau #3 · CUSTOMER kế thừa GUEST</t>
+          <t>Sau #3 · CUSTOMER kế thừa GUEST · Thực tế 5 điểm: cây kế thừa + phạm vi HUB_STAFF</t>
         </is>
       </c>
     </row>
@@ -3314,7 +4399,7 @@
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Sau #9 · CRUD, đổi vai trò, khóa và mở tài khoản</t>
+          <t>Sau #9 · CRUD, đổi vai trò, khóa và mở tài khoản · Giao diện: App Nhân viên (Expo) thay web React</t>
         </is>
       </c>
     </row>
@@ -3352,7 +4437,7 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>Sau #2 · Một quận hoặc huyện chỉ thuộc một tuyến</t>
+          <t>Sau #2 · Một quận hoặc huyện chỉ thuộc một tuyến · Giao diện: App Nhân viên (Expo) thay web React</t>
         </is>
       </c>
     </row>
@@ -3390,7 +4475,7 @@
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Sau #2 · Hai loại: gửi thường và gửi nhanh</t>
+          <t>Sau #2 · Hai loại: gửi thường và gửi nhanh · Giao diện: App Nhân viên (Expo) thay web React</t>
         </is>
       </c>
     </row>
@@ -3433,16 +4518,14 @@
       <c r="F21" s="41" t="n">
         <v>46294</v>
       </c>
-      <c r="G21" s="41" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H21" s="41" t="n">
-        <v>46294</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="J21" s="13" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="41" t="n"/>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>29/10/2026: CHƯA THỰC HIỆN — chuyển từ Sprint 2 (US-09 vượt ước lượng), chưa có mã nguồn</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28.8" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -3467,18 +4550,12 @@
       <c r="F22" s="41" t="n">
         <v>46295</v>
       </c>
-      <c r="G22" s="41" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H22" s="41" t="n">
-        <v>46295</v>
-      </c>
-      <c r="I22" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="41" t="n"/>
+      <c r="I22" s="12" t="n"/>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>Sau #11 · Mỗi điểm gắn với một khu vực phục vụ</t>
+          <t>Sau #11 · Mỗi điểm gắn với một khu vực phục vụ · 29/10/2026: chưa thực hiện</t>
         </is>
       </c>
     </row>
@@ -3505,14 +4582,12 @@
       <c r="F23" s="41" t="n">
         <v>46296</v>
       </c>
-      <c r="G23" s="41" t="n">
-        <v>46296</v>
-      </c>
+      <c r="G23" s="41" t="n"/>
       <c r="H23" s="12" t="n"/>
       <c r="I23" s="12" t="n"/>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Sau #7 ·Tự xác định khu vực từ quận hoặc huyện</t>
+          <t>Sau #7 ·Tự xác định khu vực từ quận hoặc huyện · 29/10/2026: chưa thực hiện</t>
         </is>
       </c>
     </row>
@@ -3875,12 +4950,18 @@
       <c r="F35" s="41" t="n">
         <v>46317</v>
       </c>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
+      <c r="G35" s="53" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H35" s="53" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>Sau #6 · React Native Expo · Dùng chung API xác thực với Web</t>
+          <t>Sau #6 · React Native Expo · Dùng chung API xác thực với Web · Làm sớm cùng App Nhân viên (Expo) 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -4332,13 +5413,166 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Ngoài kế hoạch Sprint — đã làm sớm (cập nhật 29/10/2026)</t>
+        </is>
+      </c>
+      <c r="B52" s="47" t="n"/>
+      <c r="C52" s="47" t="n"/>
+      <c r="D52" s="47" t="n"/>
+      <c r="E52" s="47" t="n"/>
+      <c r="F52" s="47" t="n"/>
+      <c r="G52" s="47" t="n"/>
+      <c r="H52" s="47" t="n"/>
+      <c r="I52" s="47" t="n"/>
+      <c r="J52" s="48" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>PB#1</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Xem trang chủ giới thiệu dịch vụ và vùng phục vụ (khách vãng lai)</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E53" s="41" t="n"/>
+      <c r="F53" s="41" t="n"/>
+      <c r="G53" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H53" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I53" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J53" s="13" t="inlineStr">
+        <is>
+          <t>API công khai + Web Khách hàng + App Khách hàng mobile; tìm kiếm không dấu (29/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>PB#4</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Xem bảng giá dịch vụ theo khu vực (khách vãng lai)</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E54" s="41" t="n"/>
+      <c r="F54" s="41" t="n"/>
+      <c r="G54" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H54" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I54" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>Chỉ xem; quản trị bảng giá vẫn là US-13 (Sprint 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>App Khách hàng mobile (Expo) cùng thiết kế Web Khách hàng</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n"/>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E55" s="41" t="n"/>
+      <c r="F55" s="41" t="n"/>
+      <c r="G55" s="41" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H55" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>Cổng 8083; 8 flow Maestro trên máy ảo Android (29/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Dữ liệu tự làm mới 30 giây, cache 30 giây (API Redis + app)</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E56" s="41" t="n"/>
+      <c r="F56" s="41" t="n"/>
+      <c r="G56" s="41" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H56" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="13" t="inlineStr">
+        <is>
+          <t>Yêu cầu ngày 28/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A45:J45"/>
     <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A45:J45"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A52:J52"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="E3:F3"/>

</xml_diff>

<commit_message>
docs: PERT toan du an va cap nhat Sprint Planning, Review, Retrospective, Product Backlog theo PERT
PERT viet mot lan cho Sprint 1-6: moi Sprint = phan tich + cong viec + kiem thu + du phong (1,65 sigma), mot nguoi lam nen duong gang la ca chuoi. Quy tac tre han: dung du phong, het thi keo dai Sprint va doi Sprint sau, khong cat viec. Sprint 2 keo dai den 30/10/2026, US-13 hoan thanh trong Sprint 2; Sprint 3 bat dau 02/11/2026, du an ket thuc 19/01/2027. Bo PERT cu chi co Sprint 1-2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ProductBacklog-nhom17.xlsx
+++ b/docs/ProductBacklog-nhom17.xlsx
@@ -21,9 +21,9 @@
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -726,7 +726,7 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyAlignment="1">
@@ -735,7 +735,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyAlignment="1">
@@ -872,7 +872,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -966,9 +966,10 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1540,7 +1541,7 @@
         <v>46268</v>
       </c>
       <c r="F4" s="41" t="n">
-        <v>46346</v>
+        <v>46406</v>
       </c>
     </row>
     <row r="5" ht="14.4" customHeight="1">
@@ -1566,7 +1567,7 @@
         <v>46268</v>
       </c>
       <c r="F5" s="41" t="n">
-        <v>46346</v>
+        <v>46406</v>
       </c>
     </row>
     <row r="6" ht="14.4" customHeight="1">
@@ -1592,7 +1593,7 @@
         <v>46268</v>
       </c>
       <c r="F6" s="41" t="n">
-        <v>46346</v>
+        <v>46406</v>
       </c>
     </row>
     <row r="7" ht="14.4" customHeight="1">
@@ -1618,7 +1619,7 @@
         <v>46268</v>
       </c>
       <c r="F7" s="41" t="n">
-        <v>46346</v>
+        <v>46406</v>
       </c>
     </row>
     <row r="8">
@@ -2509,7 +2510,7 @@
       </c>
       <c r="E37" s="51" t="inlineStr">
         <is>
-          <t>Done (làm sớm 22/10)</t>
+          <t>Done (làm sớm ở Sprint 2)</t>
         </is>
       </c>
       <c r="F37" s="51" t="n"/>
@@ -3472,12 +3473,12 @@
       </c>
       <c r="D75" s="24" t="inlineStr">
         <is>
-          <t>US-13 · Sprint 3</t>
+          <t>US-13 · Sprint 2</t>
         </is>
       </c>
       <c r="E75" s="51" t="inlineStr">
         <is>
-          <t>To Do (chuyển từ Sprint 2)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F75" s="51" t="n"/>
@@ -3898,11 +3899,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.861111111111111" defaultRowHeight="13.2"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="6.12962962962963" customWidth="1" min="3" max="3"/>
     <col width="12.8611111111111" customWidth="1" min="4" max="4"/>
     <col width="11.3981481481481" customWidth="1" style="39" min="5" max="5"/>
@@ -3910,7 +3911,7 @@
     <col width="14.3981481481481" customWidth="1" style="39" min="7" max="7"/>
     <col width="13.3981481481481" customWidth="1" style="39" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="35.4444444444444" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34.5" customHeight="1">
@@ -3988,32 +3989,56 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="42" t="n"/>
-      <c r="F5" s="42" t="n"/>
-      <c r="G5" s="42" t="n"/>
-      <c r="H5" s="42" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1 · 03/09/2026 – 16/09/2026 · Nền móng kỹ thuật · 10 ngày (PT 1 · DP 1,50)</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="48" t="n"/>
     </row>
     <row r="6" ht="14.4" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 1 · 03/09/2026 – 11/09/2026 · Nền móng kỹ thuật</t>
-        </is>
-      </c>
-      <c r="B6" s="47" t="n"/>
-      <c r="C6" s="47" t="n"/>
-      <c r="D6" s="47" t="n"/>
-      <c r="E6" s="47" t="n"/>
-      <c r="F6" s="47" t="n"/>
-      <c r="G6" s="47" t="n"/>
-      <c r="H6" s="47" t="n"/>
-      <c r="I6" s="47" t="n"/>
-      <c r="J6" s="48" t="n"/>
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PT1</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="n">
+        <v>46268</v>
+      </c>
+      <c r="F6" s="41" t="n">
+        <v>46268</v>
+      </c>
+      <c r="G6" s="41" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H6" s="41" t="n">
+        <v>46268</v>
+      </c>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Ngày phân tích theo PERT</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28.8" customHeight="1">
       <c r="A7" s="12" t="n">
@@ -4033,21 +4058,21 @@
         </is>
       </c>
       <c r="E7" s="41" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="F7" s="41" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>46269</v>
       </c>
-      <c r="G7" s="41" t="n">
-        <v>46268</v>
-      </c>
       <c r="H7" s="41" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="I7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="13" t="n"/>
+      <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -4067,23 +4092,23 @@
         </is>
       </c>
       <c r="E8" s="41" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="F8" s="41" t="n">
+        <v>46275</v>
+      </c>
+      <c r="G8" s="41" t="n">
         <v>46273</v>
       </c>
-      <c r="G8" s="41" t="n">
-        <v>46272</v>
-      </c>
       <c r="H8" s="41" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="I8" s="12" t="n">
         <v>6</v>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sau #1 · </t>
+          <t>Sau #1 · Vượt 1 điểm (+0,5 ngày), nằm trong dự phòng</t>
         </is>
       </c>
     </row>
@@ -4105,16 +4130,16 @@
         </is>
       </c>
       <c r="E9" s="41" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="F9" s="41" t="n">
-        <v>46275</v>
+        <v>46279</v>
       </c>
       <c r="G9" s="41" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="H9" s="41" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="I9" s="12" t="n">
         <v>5</v>
@@ -4143,16 +4168,16 @@
         </is>
       </c>
       <c r="E10" s="41" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="F10" s="41" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="G10" s="41" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="H10" s="41" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="I10" s="12" t="n">
         <v>3</v>
@@ -4164,142 +4189,136 @@
       </c>
     </row>
     <row r="11" ht="14.4" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 2 · 14/09/2026 – 25/09/2026 · Tài khoản, phân quyền và danh mục nền</t>
-        </is>
-      </c>
-      <c r="B11" s="47" t="n"/>
-      <c r="C11" s="47" t="n"/>
-      <c r="D11" s="47" t="n"/>
-      <c r="E11" s="47" t="n"/>
-      <c r="F11" s="47" t="n"/>
-      <c r="G11" s="47" t="n"/>
-      <c r="H11" s="47" t="n"/>
-      <c r="I11" s="47" t="n"/>
-      <c r="J11" s="48" t="n"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>KT1</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Viết test case, kiểm thử tích hợp và đẩy lên Git</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>46280</v>
+      </c>
+      <c r="F11" s="41" t="n">
+        <v>46280</v>
+      </c>
+      <c r="G11" s="41" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H11" s="41" t="n">
+        <v>46280</v>
+      </c>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Kiểm thử tích hợp</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28.8" customHeight="1">
-      <c r="A12" s="12" t="n">
-        <v>5</v>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>DP1</t>
+        </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Thiết lập CI pipeline tự động kiểm thử và build</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>2</v>
-      </c>
+          <t>Dự phòng 1,50 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n"/>
       <c r="D12" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
       <c r="E12" s="41" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="F12" s="41" t="n">
-        <v>46279</v>
-      </c>
-      <c r="G12" s="41" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H12" s="41" t="n">
-        <v>46279</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="13" t="n"/>
+        <v>46281</v>
+      </c>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>Dùng 0,5 ngày cho US-02</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="14.4" customHeight="1">
-      <c r="A13" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Đăng nhập hệ thống</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 2 · kế hoạch 17/09/2026 – 06/10/2026 (14 ngày, PT 1 · DP 1,75) · thực tế kéo dài đến 30/10/2026, không cắt việc · Tài khoản, phân quyền và danh mục nền</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="n"/>
+      <c r="C13" s="47" t="n"/>
+      <c r="D13" s="47" t="n"/>
+      <c r="E13" s="54" t="n"/>
+      <c r="F13" s="54" t="n"/>
+      <c r="G13" s="54" t="n"/>
+      <c r="H13" s="54" t="n"/>
+      <c r="I13" s="47" t="n"/>
+      <c r="J13" s="48" t="n"/>
+    </row>
+    <row r="14" ht="28.8" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>PT2</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E13" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="F13" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G13" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H13" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>Sau #3 ·   Khóa 15 phút sau 5 lần sai</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28.8" customHeight="1">
-      <c r="A14" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Đăng ký tài khoản khách hàng</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>DEV 1</t>
-        </is>
-      </c>
       <c r="E14" s="41" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="F14" s="41" t="n">
         <v>46282</v>
       </c>
       <c r="G14" s="41" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H14" s="41" t="n">
         <v>46282</v>
       </c>
-      <c r="I14" s="12" t="n">
-        <v>3</v>
-      </c>
+      <c r="I14" s="12" t="n"/>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Sau #6 · Tài khoản doanh nghiệp ở trạng thái PENDING chờ duyệt</t>
+          <t>Ngày phân tích theo PERT</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28.8" customHeight="1">
       <c r="A15" s="12" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Đăng xuất khỏi hệ thống</t>
+          <t>Thiết lập CI pipeline tự động kiểm thử và build</t>
         </is>
       </c>
       <c r="C15" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
@@ -4307,10 +4326,10 @@
         </is>
       </c>
       <c r="E15" s="41" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="F15" s="41" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="G15" s="41" t="n">
         <v>46283</v>
@@ -4319,25 +4338,21 @@
         <v>46283</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
-        <is>
-          <t>Sau #6 · Redis blacklist · TTL bằng hạn còn lại của Refresh Token</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
     </row>
     <row r="16" ht="14.4" customHeight="1">
       <c r="A16" s="12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Phân quyền truy cập theo vai trò</t>
+          <t>Đăng nhập hệ thống</t>
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
@@ -4354,24 +4369,24 @@
         <v>46283</v>
       </c>
       <c r="H16" s="41" t="n">
-        <v>46287</v>
+        <v>46317</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Sau #3 · CUSTOMER kế thừa GUEST · Thực tế 5 điểm: cây kế thừa + phạm vi HUB_STAFF</t>
+          <t>Sau #3 ·   Khóa 15 phút sau 5 lần sai · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="12" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Quản lý tài khoản người dùng trong hệ thống</t>
+          <t>Đăng ký tài khoản khách hàng</t>
         </is>
       </c>
       <c r="C17" s="12" t="n">
@@ -4389,31 +4404,31 @@
         <v>46287</v>
       </c>
       <c r="G17" s="41" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="H17" s="41" t="n">
-        <v>46288</v>
+        <v>46317</v>
       </c>
       <c r="I17" s="12" t="n">
         <v>3</v>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Sau #9 · CRUD, đổi vai trò, khóa và mở tài khoản · Giao diện: App Nhân viên (Expo) thay web React</t>
+          <t>Sau #6 · Tài khoản doanh nghiệp ở trạng thái PENDING chờ duyệt · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28.8" customHeight="1">
       <c r="A18" s="12" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Quản lý danh mục tuyến và khu vực phục vụ</t>
+          <t>Đăng xuất khỏi hệ thống</t>
         </is>
       </c>
       <c r="C18" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
@@ -4427,31 +4442,31 @@
         <v>46288</v>
       </c>
       <c r="G18" s="41" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="H18" s="41" t="n">
-        <v>46289</v>
+        <v>46317</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>Sau #2 · Một quận hoặc huyện chỉ thuộc một tuyến · Giao diện: App Nhân viên (Expo) thay web React</t>
+          <t>Sau #6 · Redis blacklist · TTL bằng hạn còn lại của Refresh Token · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28.8" customHeight="1">
       <c r="A19" s="12" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Quản lý danh mục loại dịch vụ vận chuyển</t>
+          <t>Phân quyền truy cập theo vai trò</t>
         </is>
       </c>
       <c r="C19" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
@@ -4459,53 +4474,75 @@
         </is>
       </c>
       <c r="E19" s="41" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="F19" s="41" t="n">
         <v>46289</v>
       </c>
       <c r="G19" s="41" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="H19" s="41" t="n">
         <v>46290</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Sau #2 · Hai loại: gửi thường và gửi nhanh · Giao diện: App Nhân viên (Expo) thay web React</t>
+          <t>Sau #3 · CUSTOMER kế thừa GUEST · Vượt 2 điểm (+1 ngày): cây kế thừa + phạm vi HUB_STAFF</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14.4" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 3 · 28/09/2026 – 09/10/2026 · Bảng giá, định giá và tạo đơn hàng</t>
-        </is>
-      </c>
-      <c r="B20" s="47" t="n"/>
-      <c r="C20" s="47" t="n"/>
-      <c r="D20" s="47" t="n"/>
-      <c r="E20" s="47" t="n"/>
-      <c r="F20" s="47" t="n"/>
-      <c r="G20" s="47" t="n"/>
-      <c r="H20" s="47" t="n"/>
-      <c r="I20" s="47" t="n"/>
-      <c r="J20" s="48" t="n"/>
+      <c r="A20" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Quản lý tài khoản người dùng trong hệ thống</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="n">
+        <v>46289</v>
+      </c>
+      <c r="F20" s="41" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G20" s="41" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H20" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>Sau #9 · CRUD, đổi vai trò, khóa và mở tài khoản · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="28.8" customHeight="1">
       <c r="A21" s="12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Quản lý bảng giá vận chuyển theo khu vực và khối lượng</t>
+          <t>Quản lý danh mục tuyến và khu vực phục vụ</t>
         </is>
       </c>
       <c r="C21" s="12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
@@ -4518,22 +4555,28 @@
       <c r="F21" s="41" t="n">
         <v>46294</v>
       </c>
-      <c r="G21" s="41" t="n"/>
-      <c r="H21" s="41" t="n"/>
-      <c r="I21" s="12" t="n"/>
+      <c r="G21" s="41" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H21" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>3</v>
+      </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>29/10/2026: CHƯA THỰC HIỆN — chuyển từ Sprint 2 (US-09 vượt ước lượng), chưa có mã nguồn</t>
+          <t>Sau #2 · Một quận hoặc huyện chỉ thuộc một tuyến · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28.8" customHeight="1">
       <c r="A22" s="12" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>Quản lý danh mục điểm tập kết và bưu cục</t>
+          <t>Quản lý danh mục loại dịch vụ vận chuyển</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
@@ -4545,31 +4588,37 @@
         </is>
       </c>
       <c r="E22" s="41" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F22" s="41" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G22" s="41" t="n">
         <v>46295</v>
       </c>
-      <c r="F22" s="41" t="n">
-        <v>46295</v>
-      </c>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="41" t="n"/>
-      <c r="I22" s="12" t="n"/>
+      <c r="H22" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>Sau #11 · Mỗi điểm gắn với một khu vực phục vụ · 29/10/2026: chưa thực hiện</t>
+          <t>Sau #2 · Hai loại: gửi thường và gửi nhanh · API xong theo lịch; giao diện hoàn thiện 22/10/2026 (App Nhân viên Expo / Web Khách hàng)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28.8" customHeight="1">
       <c r="A23" s="12" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Quản lý danh sách địa điểm lấy hàng</t>
+          <t>Quản lý bảng giá vận chuyển theo khu vực và khối lượng</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -4577,32 +4626,38 @@
         </is>
       </c>
       <c r="E23" s="41" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="F23" s="41" t="n">
-        <v>46296</v>
-      </c>
-      <c r="G23" s="41" t="n"/>
-      <c r="H23" s="12" t="n"/>
-      <c r="I23" s="12" t="n"/>
+        <v>46297</v>
+      </c>
+      <c r="G23" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="H23" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Sau #7 ·Tự xác định khu vực từ quận hoặc huyện · 29/10/2026: chưa thực hiện</t>
+          <t>Hoàn thành trong thời gian kéo dài của Sprint 2, không lùi sang Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28.8" customHeight="1">
-      <c r="A24" s="12" t="n">
-        <v>16</v>
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>KT2</t>
+        </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Ước tính phí vận chuyển trước khi gửi hàng</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="n">
-        <v>3</v>
-      </c>
+          <t>Viết test case, kiểm thử tích hợp toàn Sprint và đẩy lên GitHub</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n"/>
       <c r="D24" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
@@ -4612,29 +4667,33 @@
         <v>46297</v>
       </c>
       <c r="F24" s="41" t="n">
-        <v>46297</v>
-      </c>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="12" t="n"/>
+        <v>46300</v>
+      </c>
+      <c r="G24" s="41" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H24" s="41" t="n">
+        <v>46324</v>
+      </c>
       <c r="I24" s="12" t="n"/>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>Sau #13 ·</t>
+          <t>Kiểm thử tích hợp</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28.8" customHeight="1">
-      <c r="A25" s="12" t="n">
-        <v>17</v>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>DP2</t>
+        </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Xem phí vận chuyển dự kiến trước khi xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>5</v>
-      </c>
+          <t>Dự phòng 1,75 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n"/>
       <c r="D25" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
@@ -4646,106 +4705,106 @@
       <c r="F25" s="41" t="n">
         <v>46301</v>
       </c>
-      <c r="G25" s="12" t="n"/>
-      <c r="H25" s="12" t="n"/>
+      <c r="G25" s="41" t="n"/>
+      <c r="H25" s="41" t="n"/>
       <c r="I25" s="12" t="n"/>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Sau #13 · Khóa phí vào đơn khi xác nhận, không đổi theo bảng giá sau đó</t>
+          <t>Dùng hết (US-09); kéo dài Sprint 07/10 – 30/10/2026</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28.8" customHeight="1">
-      <c r="A26" s="12" t="n">
-        <v>18</v>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Tạo đơn hàng giao mới</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 3 · 02/11/2026 – 18/11/2026 · Định giá và tạo đơn hàng · 13 ngày (PT 1 · DP 1,75) · lịch cơ sở 07/10/2026 – 23/10/2026, dời theo quy tắc trễ hạn</t>
+        </is>
+      </c>
+      <c r="B26" s="47" t="n"/>
+      <c r="C26" s="47" t="n"/>
+      <c r="D26" s="47" t="n"/>
+      <c r="E26" s="54" t="n"/>
+      <c r="F26" s="54" t="n"/>
+      <c r="G26" s="54" t="n"/>
+      <c r="H26" s="54" t="n"/>
+      <c r="I26" s="47" t="n"/>
+      <c r="J26" s="48" t="n"/>
+    </row>
+    <row r="27" ht="28.8" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>PT3</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E26" s="41" t="n">
-        <v>46302</v>
-      </c>
-      <c r="F26" s="41" t="n">
-        <v>46303</v>
-      </c>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="12" t="n"/>
-      <c r="I26" s="12" t="n"/>
-      <c r="J26" s="13" t="inlineStr">
-        <is>
-          <t>Sau #15, #17 · Transaction · Sinh mã vận đơn + 10 chữ số</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="28.8" customHeight="1">
-      <c r="A27" s="12" t="n">
-        <v>19</v>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Khai báo tiền thu hộ COD và hình thức thanh toán phí</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>DEV 1</t>
-        </is>
-      </c>
       <c r="E27" s="41" t="n">
-        <v>46304</v>
+        <v>46328</v>
       </c>
       <c r="F27" s="41" t="n">
-        <v>46304</v>
-      </c>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="12" t="n"/>
+        <v>46328</v>
+      </c>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="41" t="n"/>
       <c r="I27" s="12" t="n"/>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>Sau #18 · Ba hình thức trả phí · Chặn khấu trừ khi thu hộ nhỏ hơn phí</t>
+          <t>Ngày phân tích theo PERT</t>
         </is>
       </c>
     </row>
     <row r="28" ht="14.4" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 4 · 12/10/2026 – 23/10/2026 · Tra cứu hành trình và phân công tự động</t>
-        </is>
-      </c>
-      <c r="B28" s="47" t="n"/>
-      <c r="C28" s="47" t="n"/>
-      <c r="D28" s="47" t="n"/>
-      <c r="E28" s="47" t="n"/>
-      <c r="F28" s="47" t="n"/>
-      <c r="G28" s="47" t="n"/>
-      <c r="H28" s="47" t="n"/>
-      <c r="I28" s="47" t="n"/>
-      <c r="J28" s="48" t="n"/>
+      <c r="A28" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Quản lý danh mục điểm tập kết và bưu cục</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="n">
+        <v>46329</v>
+      </c>
+      <c r="F28" s="41" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="41" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>Sau #11 · Mỗi điểm gắn với một khu vực phục vụ</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="28.8" customHeight="1">
       <c r="A29" s="12" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Xem chi tiết đơn hàng và toàn bộ hành trình</t>
+          <t>Quản lý danh sách địa điểm lấy hàng</t>
         </is>
       </c>
       <c r="C29" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -4753,31 +4812,31 @@
         </is>
       </c>
       <c r="E29" s="41" t="n">
-        <v>46307</v>
+        <v>46330</v>
       </c>
       <c r="F29" s="41" t="n">
-        <v>46307</v>
-      </c>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="12" t="n"/>
+        <v>46331</v>
+      </c>
+      <c r="G29" s="41" t="n"/>
+      <c r="H29" s="41" t="n"/>
       <c r="I29" s="12" t="n"/>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>Sau #18 · Đọc mảng statusHistory nhúng trong document đơn</t>
+          <t>Sau #7 ·Tự xác định khu vực từ quận hoặc huyện</t>
         </is>
       </c>
     </row>
     <row r="30" ht="28.8" customHeight="1">
       <c r="A30" s="12" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Hàng đợi sự kiện và consumer ghi nhật ký /hành trình đơn</t>
+          <t>Ước tính phí vận chuyển trước khi gửi hàng</t>
         </is>
       </c>
       <c r="C30" s="12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -4785,31 +4844,31 @@
         </is>
       </c>
       <c r="E30" s="41" t="n">
-        <v>46308</v>
+        <v>46331</v>
       </c>
       <c r="F30" s="41" t="n">
-        <v>46309</v>
-      </c>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
+        <v>46332</v>
+      </c>
+      <c r="G30" s="41" t="n"/>
+      <c r="H30" s="41" t="n"/>
       <c r="I30" s="12" t="n"/>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>Sau #18 · BullMQ trên Redis · Có retry và dead-letter queue</t>
+          <t>Sau #13</t>
         </is>
       </c>
     </row>
     <row r="31" ht="28.8" customHeight="1">
       <c r="A31" s="12" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Tra cứu hành trình đơn hàng bằng mã vận đơn</t>
+          <t>Xem phí vận chuyển dự kiến trước khi xác nhận đơn</t>
         </is>
       </c>
       <c r="C31" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
@@ -4817,31 +4876,31 @@
         </is>
       </c>
       <c r="E31" s="41" t="n">
-        <v>46310</v>
+        <v>46332</v>
       </c>
       <c r="F31" s="41" t="n">
-        <v>46310</v>
-      </c>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="12" t="n"/>
+        <v>46336</v>
+      </c>
+      <c r="G31" s="41" t="n"/>
+      <c r="H31" s="41" t="n"/>
       <c r="I31" s="12" t="n"/>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Sau #21  ·</t>
+          <t>Sau #13 · Khóa phí vào đơn khi xác nhận, không đổi theo bảng giá sau đó</t>
         </is>
       </c>
     </row>
     <row r="32" ht="28.8" customHeight="1">
       <c r="A32" s="12" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Quản lý ca làm việc và phân công nhân viên vào tuyến</t>
+          <t>Tạo đơn hàng giao mới</t>
         </is>
       </c>
       <c r="C32" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
@@ -4849,27 +4908,27 @@
         </is>
       </c>
       <c r="E32" s="41" t="n">
-        <v>46311</v>
+        <v>46336</v>
       </c>
       <c r="F32" s="41" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="12" t="n"/>
+        <v>46339</v>
+      </c>
+      <c r="G32" s="41" t="n"/>
+      <c r="H32" s="41" t="n"/>
       <c r="I32" s="12" t="n"/>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>Sau #11 · Gán người giao hàng vào tuyến theo từng ca</t>
+          <t>Sau #15, #17 · Transaction · Sinh mã vận đơn + 10 chữ số</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28.8" customHeight="1">
       <c r="A33" s="12" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình năng lực xử lý tối đa của người giao hàng</t>
+          <t>Khai báo tiền thu hộ COD và hình thức thanh toán phí</t>
         </is>
       </c>
       <c r="C33" s="12" t="n">
@@ -4881,149 +4940,143 @@
         </is>
       </c>
       <c r="E33" s="41" t="n">
-        <v>46314</v>
+        <v>46339</v>
       </c>
       <c r="F33" s="41" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G33" s="12" t="n"/>
-      <c r="H33" s="12" t="n"/>
+        <v>46342</v>
+      </c>
+      <c r="G33" s="41" t="n"/>
+      <c r="H33" s="41" t="n"/>
       <c r="I33" s="12" t="n"/>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Sau #23 · Ba cấp ưu tiên: nhân viên → tuyến → mặc định hệ thống</t>
+          <t>Sau #18 · Ba hình thức trả phí · Chặn khấu trừ khi thu hộ nhỏ hơn phí</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28.8" customHeight="1">
-      <c r="A34" s="12" t="n">
-        <v>25</v>
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>KT3</t>
+        </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Phân công đơn lấy hàng cho người giao hàng</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="n">
-        <v>5</v>
-      </c>
+          <t>Viết test case, kiểm thử end-to-end từ ước tính phí đến tạo đơn</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n"/>
       <c r="D34" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
       <c r="E34" s="41" t="n">
-        <v>46315</v>
+        <v>46342</v>
       </c>
       <c r="F34" s="41" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G34" s="12" t="n"/>
-      <c r="H34" s="12" t="n"/>
+        <v>46343</v>
+      </c>
+      <c r="G34" s="41" t="n"/>
+      <c r="H34" s="41" t="n"/>
       <c r="I34" s="12" t="n"/>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>Sau #23, #24 · Transaction chống vượt năng lực vận shipper và hàng chờ</t>
+          <t>Kiểm thử tích hợp</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28.8" customHeight="1">
-      <c r="A35" s="12" t="n">
-        <v>26</v>
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>DP3</t>
+        </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Đăng nhập ứng dụng di động</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="n">
-        <v>2</v>
-      </c>
+          <t>Dự phòng 1,75 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n"/>
       <c r="D35" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
       <c r="E35" s="41" t="n">
-        <v>46317</v>
+        <v>46343</v>
       </c>
       <c r="F35" s="41" t="n">
-        <v>46317</v>
-      </c>
-      <c r="G35" s="53" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H35" s="53" t="n">
-        <v>46317</v>
-      </c>
-      <c r="I35" s="12" t="n">
-        <v>2</v>
-      </c>
+        <v>46344</v>
+      </c>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="12" t="n"/>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>Sau #6 · React Native Expo · Dùng chung API xác thực với Web · Làm sớm cùng App Nhân viên (Expo) 22/10/2026</t>
+          <t>Chỉ dùng khi task trễ</t>
         </is>
       </c>
     </row>
     <row r="36" ht="28.8" customHeight="1">
-      <c r="A36" s="12" t="n">
-        <v>27</v>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Xem danh sách đơn cần lấy trong ca làm việc</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 4 · 19/11/2026 – 07/12/2026 · Tra cứu hành trình và phân công tự động · 13 ngày (PT 1 · DP 1,50) · lịch cơ sở 26/10/2026 – 12/11/2026, dời theo quy tắc trễ hạn</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="54" t="n"/>
+      <c r="F36" s="54" t="n"/>
+      <c r="G36" s="54" t="n"/>
+      <c r="H36" s="54" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="48" t="n"/>
+    </row>
+    <row r="37" ht="14.4" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>PT4</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E36" s="41" t="n">
-        <v>46318</v>
-      </c>
-      <c r="F36" s="41" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="12" t="n"/>
-      <c r="I36" s="12" t="n"/>
-      <c r="J36" s="13" t="inlineStr">
-        <is>
-          <t>Sau #25, #26 · Lọc theo người giao hàng và ca hiện tại</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="14.4" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 5 · 26/10/2026 – 06/11/2026 · Check-in GPS, giao hàng, thu hộ và đối soát</t>
-        </is>
-      </c>
-      <c r="B37" s="47" t="n"/>
-      <c r="C37" s="47" t="n"/>
-      <c r="D37" s="47" t="n"/>
-      <c r="E37" s="47" t="n"/>
-      <c r="F37" s="47" t="n"/>
-      <c r="G37" s="47" t="n"/>
-      <c r="H37" s="47" t="n"/>
-      <c r="I37" s="47" t="n"/>
-      <c r="J37" s="48" t="n"/>
+      <c r="E37" s="41" t="n">
+        <v>46345</v>
+      </c>
+      <c r="F37" s="41" t="n">
+        <v>46345</v>
+      </c>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="41" t="n"/>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>Ngày phân tích theo PERT</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="28.8" customHeight="1">
       <c r="A38" s="12" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Xác nhận đã lấy hàng từ người gửi</t>
+          <t>Xem chi tiết đơn hàng và toàn bộ hành trình</t>
         </is>
       </c>
       <c r="C38" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
@@ -5031,31 +5084,31 @@
         </is>
       </c>
       <c r="E38" s="41" t="n">
-        <v>46321</v>
+        <v>46346</v>
       </c>
       <c r="F38" s="41" t="n">
-        <v>46321</v>
-      </c>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="12" t="n"/>
+        <v>46346</v>
+      </c>
+      <c r="G38" s="41" t="n"/>
+      <c r="H38" s="41" t="n"/>
       <c r="I38" s="12" t="n"/>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>Sau #27 · quét mã vận đơn · Ghi tọa độ GPS và thời gian</t>
+          <t>Sau #18 · Đọc mảng statusHistory nhúng trong document đơn</t>
         </is>
       </c>
     </row>
     <row r="39" ht="28.8" customHeight="1">
       <c r="A39" s="12" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Quản lý điểm check-in trên bản đồ</t>
+          <t>Hàng đợi sự kiện và consumer ghi nhật ký /hành trình đơn</t>
         </is>
       </c>
       <c r="C39" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
@@ -5063,31 +5116,31 @@
         </is>
       </c>
       <c r="E39" s="41" t="n">
-        <v>46322</v>
+        <v>46349</v>
       </c>
       <c r="F39" s="41" t="n">
-        <v>46322</v>
-      </c>
-      <c r="G39" s="12" t="n"/>
-      <c r="H39" s="12" t="n"/>
+        <v>46351</v>
+      </c>
+      <c r="G39" s="41" t="n"/>
+      <c r="H39" s="41" t="n"/>
       <c r="I39" s="12" t="n"/>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sau #11 · Mỗi điểm gồm tọa độ và bán kính mặc định </t>
+          <t>Sau #18 · BullMQ trên Redis · Có retry và dead-letter queue</t>
         </is>
       </c>
     </row>
     <row r="40" ht="28.8" customHeight="1">
       <c r="A40" s="12" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>Tự động check-in vị trí khi đi qua điểm đã cài đặt</t>
+          <t>Tra cứu hành trình đơn hàng bằng mã vận đơn</t>
         </is>
       </c>
       <c r="C40" s="12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
@@ -5095,27 +5148,27 @@
         </is>
       </c>
       <c r="E40" s="41" t="n">
-        <v>46323</v>
+        <v>46351</v>
       </c>
       <c r="F40" s="41" t="n">
-        <v>46324</v>
-      </c>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="12" t="n"/>
+        <v>46352</v>
+      </c>
+      <c r="G40" s="41" t="n"/>
+      <c r="H40" s="41" t="n"/>
       <c r="I40" s="12" t="n"/>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Sau #29 · Chặn trùng 30 phút, hàng đợi khi mất mạng</t>
+          <t>Sau #21</t>
         </is>
       </c>
     </row>
     <row r="41" ht="28.8" customHeight="1">
       <c r="A41" s="12" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Xem danh sách đơn cần giao trong ca làm việc</t>
+          <t>Quản lý ca làm việc và phân công nhân viên vào tuyến</t>
         </is>
       </c>
       <c r="C41" s="12" t="n">
@@ -5127,27 +5180,27 @@
         </is>
       </c>
       <c r="E41" s="41" t="n">
-        <v>46325</v>
+        <v>46352</v>
       </c>
       <c r="F41" s="41" t="n">
-        <v>46325</v>
-      </c>
-      <c r="G41" s="12" t="n"/>
-      <c r="H41" s="12" t="n"/>
+        <v>46353</v>
+      </c>
+      <c r="G41" s="41" t="n"/>
+      <c r="H41" s="41" t="n"/>
       <c r="I41" s="12" t="n"/>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>Sau #25 · Lọc theo người giao hàng và ca hiện tại</t>
+          <t>Sau #11 · Gán người giao hàng vào tuyến theo từng ca</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28.8" customHeight="1">
       <c r="A42" s="12" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>Xác nhận giao hàng thành công cho người nhận</t>
+          <t>Cấu hình năng lực xử lý tối đa của người giao hàng</t>
         </is>
       </c>
       <c r="C42" s="12" t="n">
@@ -5159,31 +5212,31 @@
         </is>
       </c>
       <c r="E42" s="41" t="n">
-        <v>46328</v>
+        <v>46353</v>
       </c>
       <c r="F42" s="41" t="n">
-        <v>46328</v>
-      </c>
-      <c r="G42" s="12" t="n"/>
-      <c r="H42" s="12" t="n"/>
+        <v>46356</v>
+      </c>
+      <c r="G42" s="41" t="n"/>
+      <c r="H42" s="41" t="n"/>
       <c r="I42" s="12" t="n"/>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>Sau #31 · Ghi tọa độ GPS · Chuyển DELIVERED, không đổi trạng thái được nữa</t>
+          <t>Sau #23 · Ba cấp ưu tiên: nhân viên → tuyến → mặc định hệ thống</t>
         </is>
       </c>
     </row>
     <row r="43" ht="28.8" customHeight="1">
       <c r="A43" s="12" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>Ghi nhận đã thu tiền COD từ người nhận</t>
+          <t>Phân công đơn lấy hàng cho người giao hàng</t>
         </is>
       </c>
       <c r="C43" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
@@ -5191,207 +5244,209 @@
         </is>
       </c>
       <c r="E43" s="41" t="n">
-        <v>46329</v>
+        <v>46356</v>
       </c>
       <c r="F43" s="41" t="n">
-        <v>46330</v>
-      </c>
-      <c r="G43" s="12" t="n"/>
-      <c r="H43" s="12" t="n"/>
+        <v>46358</v>
+      </c>
+      <c r="G43" s="41" t="n"/>
+      <c r="H43" s="41" t="n"/>
       <c r="I43" s="12" t="n"/>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>Sau #32 ·  Thu tiền mặt hoặc chuyển khoản</t>
+          <t>Sau #23, #24 · Transaction chống vượt năng lực vận shipper và hàng chờ</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28.8" customHeight="1">
       <c r="A44" s="12" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Tạo đối soát và tổng hợp số liệu cho khách hàng</t>
+          <t>Đăng nhập ứng dụng di động</t>
         </is>
       </c>
       <c r="C44" s="12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E44" s="41" t="n">
-        <v>46331</v>
-      </c>
-      <c r="F44" s="41" t="n">
-        <v>46332</v>
-      </c>
-      <c r="G44" s="12" t="n"/>
-      <c r="H44" s="12" t="n"/>
-      <c r="I44" s="12" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H44" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>Sau #33 · Một đơn chỉ thuộc một kỳ đối soát</t>
+          <t>Sau #6 · React Native Expo · Dùng chung API xác thực với Web · Làm sớm cùng App Nhân viên ở Sprint 2; lịch điều chỉnh không tính lại</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 6 · 09/11/2026 – 22/11/2026 · Hoàn hàng, sự cố và thống kê (bổ sung theo case study)</t>
-        </is>
-      </c>
-      <c r="B45" s="47" t="n"/>
-      <c r="C45" s="47" t="n"/>
-      <c r="D45" s="47" t="n"/>
-      <c r="E45" s="47" t="n"/>
-      <c r="F45" s="47" t="n"/>
-      <c r="G45" s="47" t="n"/>
-      <c r="H45" s="47" t="n"/>
-      <c r="I45" s="47" t="n"/>
-      <c r="J45" s="48" t="n"/>
+      <c r="A45" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>Xem danh sách đơn cần lấy trong ca làm việc</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E45" s="41" t="n">
+        <v>46358</v>
+      </c>
+      <c r="F45" s="41" t="n">
+        <v>46359</v>
+      </c>
+      <c r="G45" s="41" t="n"/>
+      <c r="H45" s="41" t="n"/>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="13" t="inlineStr">
+        <is>
+          <t>Sau #25, #26 · Lọc theo người giao hàng và ca hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
-        <v>35</v>
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>KT4</t>
+        </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>Phân công tự động đơn giao hàng cho người giao hàng</t>
-        </is>
-      </c>
-      <c r="C46" s="12" t="n">
-        <v>5</v>
-      </c>
+          <t>Viết test case, kiểm thử tích hợp toàn Sprint và đẩy lên GitHub</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n"/>
       <c r="D46" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
       <c r="E46" s="41" t="n">
-        <v>46335</v>
+        <v>46359</v>
       </c>
       <c r="F46" s="41" t="n">
-        <v>46336</v>
+        <v>46360</v>
       </c>
       <c r="G46" s="41" t="n"/>
       <c r="H46" s="41" t="n"/>
       <c r="I46" s="12" t="n"/>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>Sau #27 · PB#52 · Thuật toán giống chiều lấy hàng, kích hoạt khi đơn đến AT_DEST_HUB</t>
+          <t>Kiểm thử tích hợp</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="n">
-        <v>36</v>
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>DP4</t>
+        </is>
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình chính sách giao lại, giới hạn số lần giao</t>
-        </is>
-      </c>
-      <c r="C47" s="12" t="n">
-        <v>2</v>
-      </c>
+          <t>Dự phòng 1,50 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n"/>
       <c r="D47" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
       <c r="E47" s="41" t="n">
-        <v>46337</v>
+        <v>46360</v>
       </c>
       <c r="F47" s="41" t="n">
-        <v>46337</v>
+        <v>46363</v>
       </c>
       <c r="G47" s="41" t="n"/>
       <c r="H47" s="41" t="n"/>
       <c r="I47" s="12" t="n"/>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>Sau #32 · PB#77 · Mặc định tối đa 3 lần giao, vượt quá chuyển RETURNING</t>
+          <t>Chỉ dùng khi task trễ</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n">
-        <v>37</v>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>Quy trình hoàn hàng — phân công theo tuyến, theo dõi đến khi shop xác nhận</t>
-        </is>
-      </c>
-      <c r="C48" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 5 · 08/12/2026 – 28/12/2026 · Lấy/giao hàng, check-in GPS, thu hộ và đối soát · 15 ngày (PT 1 · DP 2,25) · lịch cơ sở 13/11/2026 – 03/12/2026, dời theo quy tắc trễ hạn</t>
+        </is>
+      </c>
+      <c r="B48" s="47" t="n"/>
+      <c r="C48" s="47" t="n"/>
+      <c r="D48" s="47" t="n"/>
+      <c r="E48" s="54" t="n"/>
+      <c r="F48" s="54" t="n"/>
+      <c r="G48" s="54" t="n"/>
+      <c r="H48" s="54" t="n"/>
+      <c r="I48" s="47" t="n"/>
+      <c r="J48" s="48" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>PT5</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E48" s="41" t="n">
-        <v>46338</v>
-      </c>
-      <c r="F48" s="41" t="n">
-        <v>46339</v>
-      </c>
-      <c r="G48" s="41" t="n"/>
-      <c r="H48" s="41" t="n"/>
-      <c r="I48" s="12" t="n"/>
-      <c r="J48" s="13" t="inlineStr">
-        <is>
-          <t>Sau #36 · PB#43, #57 · Assignment.type=RETURN, kết thúc ở trạng thái RETURNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="n">
-        <v>38</v>
-      </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>Ghi nhận sự cố/khiếu nại, theo dõi xử lý và kết quả</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="D49" s="12" t="inlineStr">
-        <is>
-          <t>DEV 1</t>
-        </is>
-      </c>
       <c r="E49" s="41" t="n">
-        <v>46342</v>
+        <v>46364</v>
       </c>
       <c r="F49" s="41" t="n">
-        <v>46343</v>
+        <v>46364</v>
       </c>
       <c r="G49" s="41" t="n"/>
       <c r="H49" s="41" t="n"/>
       <c r="I49" s="12" t="n"/>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>PB#45, #61 · Ghi nhận được ở bất kỳ thời điểm nào trong vòng đời đơn, đơn chuyển trạng thái INCIDENT</t>
+          <t>Ngày phân tích theo PERT</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>Thống kê tổng hợp và dashboard quản trị</t>
+          <t>Xác nhận đã lấy hàng từ người gửi</t>
         </is>
       </c>
       <c r="C50" s="12" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
@@ -5399,184 +5454,868 @@
         </is>
       </c>
       <c r="E50" s="41" t="n">
-        <v>46344</v>
+        <v>46365</v>
       </c>
       <c r="F50" s="41" t="n">
-        <v>46346</v>
+        <v>46365</v>
       </c>
       <c r="G50" s="41" t="n"/>
       <c r="H50" s="41" t="n"/>
       <c r="I50" s="12" t="n"/>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>Sau #34 · PB#78–82 · Aggregation pipeline trên orders/settlements, không thêm collection mới</t>
+          <t>Sau #27 · quét mã vận đơn · Ghi tọa độ GPS và thời gian</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Quản lý điểm check-in trên bản đồ</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E51" s="41" t="n">
+        <v>46366</v>
+      </c>
+      <c r="F51" s="41" t="n">
+        <v>46366</v>
+      </c>
+      <c r="G51" s="41" t="n"/>
+      <c r="H51" s="41" t="n"/>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="13" t="inlineStr">
+        <is>
+          <t>Sau #11 · Mỗi điểm gồm tọa độ và bán kính mặc định</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="inlineStr">
-        <is>
-          <t>Ngoài kế hoạch Sprint — đã làm sớm (cập nhật 29/10/2026)</t>
-        </is>
-      </c>
-      <c r="B52" s="47" t="n"/>
-      <c r="C52" s="47" t="n"/>
-      <c r="D52" s="47" t="n"/>
-      <c r="E52" s="47" t="n"/>
-      <c r="F52" s="47" t="n"/>
-      <c r="G52" s="47" t="n"/>
-      <c r="H52" s="47" t="n"/>
-      <c r="I52" s="47" t="n"/>
-      <c r="J52" s="48" t="n"/>
+      <c r="A52" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>Tự động check-in vị trí khi đi qua điểm đã cài đặt</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E52" s="41" t="n">
+        <v>46367</v>
+      </c>
+      <c r="F52" s="41" t="n">
+        <v>46371</v>
+      </c>
+      <c r="G52" s="41" t="n"/>
+      <c r="H52" s="41" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>Sau #29 · Chặn trùng 30 phút, hàng đợi khi mất mạng</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="12" t="inlineStr">
-        <is>
-          <t>PB#1</t>
-        </is>
+      <c r="A53" s="12" t="n">
+        <v>31</v>
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>Xem trang chủ giới thiệu dịch vụ và vùng phục vụ (khách vãng lai)</t>
+          <t>Xem danh sách đơn cần giao trong ca làm việc</t>
         </is>
       </c>
       <c r="C53" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E53" s="41" t="n"/>
-      <c r="F53" s="41" t="n"/>
-      <c r="G53" s="41" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H53" s="41" t="n">
-        <v>46324</v>
-      </c>
-      <c r="I53" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="E53" s="41" t="n">
+        <v>46371</v>
+      </c>
+      <c r="F53" s="41" t="n">
+        <v>46372</v>
+      </c>
+      <c r="G53" s="41" t="n"/>
+      <c r="H53" s="41" t="n"/>
+      <c r="I53" s="12" t="n"/>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>API công khai + Web Khách hàng + App Khách hàng mobile; tìm kiếm không dấu (29/10/2026)</t>
+          <t>Sau #25 · Lọc theo người giao hàng và ca hiện tại</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="inlineStr">
-        <is>
-          <t>PB#4</t>
-        </is>
+      <c r="A54" s="12" t="n">
+        <v>32</v>
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
-          <t>Xem bảng giá dịch vụ theo khu vực (khách vãng lai)</t>
+          <t>Xác nhận giao hàng thành công cho người nhận</t>
         </is>
       </c>
       <c r="C54" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E54" s="41" t="n"/>
-      <c r="F54" s="41" t="n"/>
-      <c r="G54" s="41" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H54" s="41" t="n">
-        <v>46324</v>
-      </c>
-      <c r="I54" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="E54" s="41" t="n">
+        <v>46372</v>
+      </c>
+      <c r="F54" s="41" t="n">
+        <v>46373</v>
+      </c>
+      <c r="G54" s="41" t="n"/>
+      <c r="H54" s="41" t="n"/>
+      <c r="I54" s="12" t="n"/>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>Chỉ xem; quản trị bảng giá vẫn là US-13 (Sprint 3)</t>
+          <t>Sau #31 · Ghi tọa độ GPS · Chuyển DELIVERED, không đổi trạng thái được nữa</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="A55" s="12" t="n">
+        <v>33</v>
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>App Khách hàng mobile (Expo) cùng thiết kế Web Khách hàng</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="n"/>
+          <t>Ghi nhận đã thu tiền COD từ người nhận</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n">
+        <v>3</v>
+      </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E55" s="41" t="n"/>
-      <c r="F55" s="41" t="n"/>
-      <c r="G55" s="41" t="n">
-        <v>46323</v>
-      </c>
-      <c r="H55" s="41" t="n">
-        <v>46324</v>
-      </c>
+      <c r="E55" s="41" t="n">
+        <v>46373</v>
+      </c>
+      <c r="F55" s="41" t="n">
+        <v>46377</v>
+      </c>
+      <c r="G55" s="41" t="n"/>
+      <c r="H55" s="41" t="n"/>
       <c r="I55" s="12" t="n"/>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>Cổng 8083; 8 flow Maestro trên máy ảo Android (29/10/2026)</t>
+          <t>Sau #32 ·  Thu tiền mặt hoặc chuyển khoản</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="A56" s="12" t="n">
+        <v>34</v>
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
-          <t>Dữ liệu tự làm mới 30 giây, cache 30 giây (API Redis + app)</t>
-        </is>
-      </c>
-      <c r="C56" s="12" t="n"/>
+          <t>Tạo đối soát và tổng hợp số liệu cho khách hàng</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
           <t>DEV 1</t>
         </is>
       </c>
-      <c r="E56" s="41" t="n"/>
-      <c r="F56" s="41" t="n"/>
-      <c r="G56" s="41" t="n">
-        <v>46323</v>
-      </c>
-      <c r="H56" s="41" t="n">
-        <v>46324</v>
-      </c>
+      <c r="E56" s="41" t="n">
+        <v>46377</v>
+      </c>
+      <c r="F56" s="41" t="n">
+        <v>46379</v>
+      </c>
+      <c r="G56" s="41" t="n"/>
+      <c r="H56" s="41" t="n"/>
       <c r="I56" s="12" t="n"/>
       <c r="J56" s="13" t="inlineStr">
         <is>
+          <t>Sau #33 · Một đơn chỉ thuộc một kỳ đối soát</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>KT5</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Viết test case, kiểm thử tích hợp toàn Sprint và đẩy lên GitHub</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E57" s="41" t="n">
+        <v>46379</v>
+      </c>
+      <c r="F57" s="41" t="n">
+        <v>46380</v>
+      </c>
+      <c r="G57" s="41" t="n"/>
+      <c r="H57" s="41" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="13" t="inlineStr">
+        <is>
+          <t>Kiểm thử tích hợp</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>DP5</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>Dự phòng 2,25 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="n"/>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E58" s="41" t="n">
+        <v>46380</v>
+      </c>
+      <c r="F58" s="41" t="n">
+        <v>46384</v>
+      </c>
+      <c r="G58" s="41" t="n"/>
+      <c r="H58" s="41" t="n"/>
+      <c r="I58" s="12" t="n"/>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>Chỉ dùng khi task trễ</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 6 · 29/12/2026 – 19/01/2027 · Hoàn hàng, sự cố và thống kê · 15 ngày (PT 1 · DP 2,00) · lịch cơ sở 04/12/2026 – 24/12/2026, dời theo quy tắc trễ hạn</t>
+        </is>
+      </c>
+      <c r="B59" s="47" t="n"/>
+      <c r="C59" s="47" t="n"/>
+      <c r="D59" s="47" t="n"/>
+      <c r="E59" s="54" t="n"/>
+      <c r="F59" s="54" t="n"/>
+      <c r="G59" s="54" t="n"/>
+      <c r="H59" s="54" t="n"/>
+      <c r="I59" s="47" t="n"/>
+      <c r="J59" s="48" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>PT6</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Phân tích yêu cầu, thiết kế chi tiết, lập kế hoạch Sprint</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E60" s="41" t="n">
+        <v>46385</v>
+      </c>
+      <c r="F60" s="41" t="n">
+        <v>46385</v>
+      </c>
+      <c r="G60" s="41" t="n"/>
+      <c r="H60" s="41" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="13" t="inlineStr">
+        <is>
+          <t>Ngày phân tích theo PERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Phân công tự động đơn giao hàng cho người giao hàng</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E61" s="41" t="n">
+        <v>46386</v>
+      </c>
+      <c r="F61" s="41" t="n">
+        <v>46387</v>
+      </c>
+      <c r="G61" s="41" t="n"/>
+      <c r="H61" s="41" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>Sau #27 · PB#52 · Thuật toán giống chiều lấy hàng, kích hoạt khi đơn đến AT_DEST_HUB</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Cấu hình chính sách giao lại, giới hạn số lần giao</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E62" s="41" t="n">
+        <v>46391</v>
+      </c>
+      <c r="F62" s="41" t="n">
+        <v>46391</v>
+      </c>
+      <c r="G62" s="41" t="n"/>
+      <c r="H62" s="41" t="n"/>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="13" t="inlineStr">
+        <is>
+          <t>Sau #32 · PB#77 · Mặc định tối đa 3 lần giao, vượt quá chuyển RETURNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Quy trình hoàn hàng — phân công theo tuyến, theo dõi đến khi shop xác nhận</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E63" s="41" t="n">
+        <v>46392</v>
+      </c>
+      <c r="F63" s="41" t="n">
+        <v>46394</v>
+      </c>
+      <c r="G63" s="41" t="n"/>
+      <c r="H63" s="41" t="n"/>
+      <c r="I63" s="12" t="n"/>
+      <c r="J63" s="13" t="inlineStr">
+        <is>
+          <t>Sau #36 · PB#43, #57 · Assignment.type=RETURN, kết thúc ở trạng thái RETURNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Ghi nhận sự cố/khiếu nại, theo dõi xử lý và kết quả</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E64" s="41" t="n">
+        <v>46394</v>
+      </c>
+      <c r="F64" s="41" t="n">
+        <v>46398</v>
+      </c>
+      <c r="G64" s="41" t="n"/>
+      <c r="H64" s="41" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="13" t="inlineStr">
+        <is>
+          <t>PB#45, #61 · Ghi nhận được ở bất kỳ thời điểm nào trong vòng đời đơn, đơn chuyển trạng thái INCIDENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Thống kê tổng hợp và dashboard quản trị</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E65" s="41" t="n">
+        <v>46398</v>
+      </c>
+      <c r="F65" s="41" t="n">
+        <v>46401</v>
+      </c>
+      <c r="G65" s="41" t="n"/>
+      <c r="H65" s="41" t="n"/>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="13" t="inlineStr">
+        <is>
+          <t>Sau #34 · PB#78–82 · Aggregation pipeline trên orders/settlements, không thêm collection mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>KT6</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Kiểm thử toàn hệ thống, chuẩn bị bàn giao</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E66" s="41" t="n">
+        <v>46402</v>
+      </c>
+      <c r="F66" s="41" t="n">
+        <v>46402</v>
+      </c>
+      <c r="G66" s="41" t="n"/>
+      <c r="H66" s="41" t="n"/>
+      <c r="I66" s="12" t="n"/>
+      <c r="J66" s="13" t="inlineStr">
+        <is>
+          <t>Kiểm thử tích hợp</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>DP6</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>Dự phòng 2,00 ngày (1,65σ theo PERT)</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E67" s="41" t="n">
+        <v>46405</v>
+      </c>
+      <c r="F67" s="41" t="n">
+        <v>46406</v>
+      </c>
+      <c r="G67" s="41" t="n"/>
+      <c r="H67" s="41" t="n"/>
+      <c r="I67" s="12" t="n"/>
+      <c r="J67" s="13" t="inlineStr">
+        <is>
+          <t>Chỉ dùng khi task trễ</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Ngoài kế hoạch Sprint — đã làm sớm (cập nhật 29/10/2026)</t>
+        </is>
+      </c>
+      <c r="B68" s="47" t="n"/>
+      <c r="C68" s="47" t="n"/>
+      <c r="D68" s="47" t="n"/>
+      <c r="E68" s="54" t="n"/>
+      <c r="F68" s="54" t="n"/>
+      <c r="G68" s="54" t="n"/>
+      <c r="H68" s="54" t="n"/>
+      <c r="I68" s="47" t="n"/>
+      <c r="J68" s="48" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>PB#1</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>Xem trang chủ giới thiệu dịch vụ và vùng phục vụ (khách vãng lai)</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E69" s="41" t="n"/>
+      <c r="F69" s="41" t="n"/>
+      <c r="G69" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H69" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I69" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>API công khai + Web Khách hàng + App Khách hàng mobile; tìm kiếm không dấu</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>PB#4</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>Xem bảng giá dịch vụ theo khu vực (khách vãng lai)</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E70" s="41" t="n"/>
+      <c r="F70" s="41" t="n"/>
+      <c r="G70" s="41" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H70" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I70" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>Chỉ xem; quản trị bảng giá là US-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>App Khách hàng mobile (Expo) cùng thiết kế Web Khách hàng</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="n"/>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E71" s="41" t="n"/>
+      <c r="F71" s="41" t="n"/>
+      <c r="G71" s="41" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H71" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I71" s="12" t="n"/>
+      <c r="J71" s="13" t="inlineStr">
+        <is>
+          <t>8 flow Maestro trên máy ảo Android</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>Dữ liệu tự làm mới 30 giây, cache 30 giây (API Redis + app)</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="n"/>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>DEV 1</t>
+        </is>
+      </c>
+      <c r="E72" s="41" t="n"/>
+      <c r="F72" s="41" t="n"/>
+      <c r="G72" s="41" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H72" s="41" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I72" s="12" t="n"/>
+      <c r="J72" s="13" t="inlineStr">
+        <is>
           <t>Yêu cầu ngày 28/10/2026</t>
         </is>
       </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="n"/>
+      <c r="B73" s="13" t="n"/>
+      <c r="C73" s="12" t="n"/>
+      <c r="D73" s="12" t="n"/>
+      <c r="E73" s="41" t="n"/>
+      <c r="F73" s="41" t="n"/>
+      <c r="G73" s="41" t="n"/>
+      <c r="H73" s="41" t="n"/>
+      <c r="I73" s="12" t="n"/>
+      <c r="J73" s="13" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="n"/>
+      <c r="B74" s="13" t="n"/>
+      <c r="C74" s="12" t="n"/>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="41" t="n"/>
+      <c r="F74" s="41" t="n"/>
+      <c r="G74" s="41" t="n"/>
+      <c r="H74" s="41" t="n"/>
+      <c r="I74" s="12" t="n"/>
+      <c r="J74" s="13" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="n"/>
+      <c r="B75" s="13" t="n"/>
+      <c r="C75" s="12" t="n"/>
+      <c r="D75" s="12" t="n"/>
+      <c r="E75" s="41" t="n"/>
+      <c r="F75" s="41" t="n"/>
+      <c r="G75" s="41" t="n"/>
+      <c r="H75" s="41" t="n"/>
+      <c r="I75" s="12" t="n"/>
+      <c r="J75" s="13" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="n"/>
+      <c r="B76" s="13" t="n"/>
+      <c r="C76" s="12" t="n"/>
+      <c r="D76" s="12" t="n"/>
+      <c r="E76" s="41" t="n"/>
+      <c r="F76" s="41" t="n"/>
+      <c r="G76" s="41" t="n"/>
+      <c r="H76" s="41" t="n"/>
+      <c r="I76" s="12" t="n"/>
+      <c r="J76" s="13" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="n"/>
+      <c r="B77" s="13" t="n"/>
+      <c r="C77" s="12" t="n"/>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="41" t="n"/>
+      <c r="F77" s="41" t="n"/>
+      <c r="G77" s="41" t="n"/>
+      <c r="H77" s="41" t="n"/>
+      <c r="I77" s="12" t="n"/>
+      <c r="J77" s="13" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="n"/>
+      <c r="B78" s="13" t="n"/>
+      <c r="C78" s="12" t="n"/>
+      <c r="D78" s="12" t="n"/>
+      <c r="E78" s="41" t="n"/>
+      <c r="F78" s="41" t="n"/>
+      <c r="G78" s="41" t="n"/>
+      <c r="H78" s="41" t="n"/>
+      <c r="I78" s="12" t="n"/>
+      <c r="J78" s="13" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="n"/>
+      <c r="B79" s="13" t="n"/>
+      <c r="C79" s="12" t="n"/>
+      <c r="D79" s="12" t="n"/>
+      <c r="E79" s="41" t="n"/>
+      <c r="F79" s="41" t="n"/>
+      <c r="G79" s="41" t="n"/>
+      <c r="H79" s="41" t="n"/>
+      <c r="I79" s="12" t="n"/>
+      <c r="J79" s="13" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="n"/>
+      <c r="B80" s="13" t="n"/>
+      <c r="C80" s="12" t="n"/>
+      <c r="D80" s="12" t="n"/>
+      <c r="E80" s="41" t="n"/>
+      <c r="F80" s="41" t="n"/>
+      <c r="G80" s="41" t="n"/>
+      <c r="H80" s="41" t="n"/>
+      <c r="I80" s="12" t="n"/>
+      <c r="J80" s="13" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="n"/>
+      <c r="B81" s="13" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="12" t="n"/>
+      <c r="E81" s="41" t="n"/>
+      <c r="F81" s="41" t="n"/>
+      <c r="G81" s="41" t="n"/>
+      <c r="H81" s="41" t="n"/>
+      <c r="I81" s="12" t="n"/>
+      <c r="J81" s="13" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="n"/>
+      <c r="B82" s="13" t="n"/>
+      <c r="C82" s="12" t="n"/>
+      <c r="D82" s="12" t="n"/>
+      <c r="E82" s="41" t="n"/>
+      <c r="F82" s="41" t="n"/>
+      <c r="G82" s="41" t="n"/>
+      <c r="H82" s="41" t="n"/>
+      <c r="I82" s="12" t="n"/>
+      <c r="J82" s="13" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="n"/>
+      <c r="B83" s="13" t="n"/>
+      <c r="C83" s="12" t="n"/>
+      <c r="D83" s="12" t="n"/>
+      <c r="E83" s="41" t="n"/>
+      <c r="F83" s="41" t="n"/>
+      <c r="G83" s="41" t="n"/>
+      <c r="H83" s="41" t="n"/>
+      <c r="I83" s="12" t="n"/>
+      <c r="J83" s="13" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="n"/>
+      <c r="B84" s="13" t="n"/>
+      <c r="C84" s="12" t="n"/>
+      <c r="D84" s="12" t="n"/>
+      <c r="E84" s="41" t="n"/>
+      <c r="F84" s="41" t="n"/>
+      <c r="G84" s="41" t="n"/>
+      <c r="H84" s="41" t="n"/>
+      <c r="I84" s="12" t="n"/>
+      <c r="J84" s="13" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="n"/>
+      <c r="B85" s="13" t="n"/>
+      <c r="C85" s="12" t="n"/>
+      <c r="D85" s="12" t="n"/>
+      <c r="E85" s="41" t="n"/>
+      <c r="F85" s="41" t="n"/>
+      <c r="G85" s="41" t="n"/>
+      <c r="H85" s="41" t="n"/>
+      <c r="I85" s="12" t="n"/>
+      <c r="J85" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A45:J45"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A52:J52"/>
-    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A59:J59"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A68:J68"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A13:J13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>